<commit_message>
Add questions: Question Bank
</commit_message>
<xml_diff>
--- a/surveys/question-bank/questions.xlsx
+++ b/surveys/question-bank/questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mhaight\Python\InterviewGuides\surveys\question-bank\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103AE846-16EC-4A77-9225-403F12EAC80E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A645C571-2633-42E2-8EBD-A9D1488F7F9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="10785" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,9 +38,6 @@
     <t>Guide URL</t>
   </si>
   <si>
-    <t>Interview Guide 1</t>
-  </si>
-  <si>
     <t>Category</t>
   </si>
   <si>
@@ -138,6 +135,9 @@
   </si>
   <si>
     <t>Test Survey</t>
+  </si>
+  <si>
+    <t>Interview Guide</t>
   </si>
 </sst>
 </file>
@@ -233,6 +233,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -240,7 +241,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -552,25 +552,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
+      <c r="B1" s="6"/>
     </row>
     <row r="2" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="10" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:2" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5"/>
+      <c r="B4" s="6"/>
     </row>
     <row r="5" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
@@ -582,10 +582,10 @@
     </row>
     <row r="6" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -612,217 +612,217 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
         <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
         <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" t="s">
         <v>30</v>
-      </c>
-      <c r="B20" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>